<commit_message>
TPRO-16: feat: add skipline feature and update test data with latest format
</commit_message>
<xml_diff>
--- a/src/test/resources/sample/2023-07-boc.xlsx
+++ b/src/test/resources/sample/2023-07-boc.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\java\transaction-hub\transaction-processor\src\test\resources\sample\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{504110E3-6622-4348-9217-E557C2766D75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D29F46EB-176A-40A7-9076-798BD159EBAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{2E4299CF-EAEC-4051-BBF4-A6C80EEB9106}"/>
   </bookViews>
@@ -20,25 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
-  <si>
-    <t>Date</t>
-  </si>
-  <si>
-    <t>Transaction Details</t>
-  </si>
-  <si>
-    <t>Deposit</t>
-  </si>
-  <si>
-    <t>Withdrawal</t>
-  </si>
-  <si>
-    <t>Balance in Original Currency</t>
-  </si>
-  <si>
-    <t>Balance Brought Forward</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>Transfer FPS/PO LEUNG KUK/12230725F280350081</t>
   </si>
@@ -49,7 +31,19 @@
     <t>Transfer FPS/MR CHAN TAI MAN/FRN20230725PAYC0101333496718</t>
   </si>
   <si>
-    <t>Balance Carried Forward</t>
+    <t>Transaction Date</t>
+  </si>
+  <si>
+    <t>Withdrawals</t>
+  </si>
+  <si>
+    <t>Deposits</t>
+  </si>
+  <si>
+    <t>Balance/Debit(DR)</t>
+  </si>
+  <si>
+    <t>Particulars</t>
   </si>
 </sst>
 </file>
@@ -603,14 +597,14 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2E173E32-1B9D-4D52-8D80-46894537BB26}" name="Table1" displayName="Table1" ref="A1:E6" totalsRowShown="0">
-  <autoFilter ref="A1:E6" xr:uid="{2E173E32-1B9D-4D52-8D80-46894537BB26}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2E173E32-1B9D-4D52-8D80-46894537BB26}" name="Table1" displayName="Table1" ref="A1:E4" totalsRowShown="0">
+  <autoFilter ref="A1:E4" xr:uid="{2E173E32-1B9D-4D52-8D80-46894537BB26}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{5DEFFFB9-A937-42FC-9AF0-C5E1A1671AB0}" name="Date" dataDxfId="1"/>
-    <tableColumn id="2" xr3:uid="{ED9EF2F9-1650-4320-96F3-7EAC5B19F876}" name="Transaction Details"/>
-    <tableColumn id="3" xr3:uid="{4DE0488B-DF31-4F3E-933F-ABDF37077624}" name="Deposit"/>
-    <tableColumn id="4" xr3:uid="{E2267EA2-A141-4A1A-BA94-429F43A0733E}" name="Withdrawal"/>
-    <tableColumn id="5" xr3:uid="{EDF115DB-F61F-472D-8579-36BE371DE78C}" name="Balance in Original Currency" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{5DEFFFB9-A937-42FC-9AF0-C5E1A1671AB0}" name="Transaction Date" dataDxfId="1"/>
+    <tableColumn id="2" xr3:uid="{ED9EF2F9-1650-4320-96F3-7EAC5B19F876}" name="Particulars"/>
+    <tableColumn id="3" xr3:uid="{4DE0488B-DF31-4F3E-933F-ABDF37077624}" name="Deposits"/>
+    <tableColumn id="4" xr3:uid="{E2267EA2-A141-4A1A-BA94-429F43A0733E}" name="Withdrawals"/>
+    <tableColumn id="5" xr3:uid="{EDF115DB-F61F-472D-8579-36BE371DE78C}" name="Balance/Debit(DR)" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -933,10 +927,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DBAEDEE3-053E-4027-B257-283F20B4FFB0}">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.5703125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="59.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="8.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11.140625" bestFit="1" customWidth="1"/>
@@ -945,30 +939,33 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C1" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E1" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
-        <v>45107</v>
+        <v>45132</v>
       </c>
       <c r="B2" t="s">
-        <v>5</v>
+        <v>0</v>
+      </c>
+      <c r="D2" s="2">
+        <v>3000</v>
       </c>
       <c r="E2" s="2">
-        <v>4000</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -976,13 +973,13 @@
         <v>45132</v>
       </c>
       <c r="B3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D3" s="2">
-        <v>3000</v>
-      </c>
-      <c r="E3" s="2">
-        <v>1000</v>
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>500</v>
+      </c>
+      <c r="E3">
+        <v>500</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -990,37 +987,12 @@
         <v>45132</v>
       </c>
       <c r="B4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D4">
-        <v>500</v>
-      </c>
-      <c r="E4">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="1">
-        <v>45132</v>
-      </c>
-      <c r="B5" t="s">
-        <v>8</v>
-      </c>
-      <c r="C5" s="2">
+        <v>2</v>
+      </c>
+      <c r="C4" s="2">
         <v>3500</v>
       </c>
-      <c r="E5" s="2">
-        <v>4000</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="1">
-        <v>45138</v>
-      </c>
-      <c r="B6" t="s">
-        <v>9</v>
-      </c>
-      <c r="E6" s="2">
+      <c r="E4" s="2">
         <v>4000</v>
       </c>
     </row>

</xml_diff>